<commit_message>
Updated energy analysis plots with cumulative line for affected wrist and strokenet_wrist.py finds optimal thresholds
</commit_message>
<xml_diff>
--- a/outputs/results/subject_energy/Hub_test_energy.xlsx
+++ b/outputs/results/subject_energy/Hub_test_energy.xlsx
@@ -21256,7 +21256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21286,292 +21286,344 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Affected wrist</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Target non-walk energy (affected)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Affected wrist non-walk energy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>75243.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Target achieved</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Recording start</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>11/03/2026 12:18:19</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Recording end</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>11/03/2026 12:25:46</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Total windows</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B10" t="n">
         <v>629</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Walking windows</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B11" t="n">
         <v>177</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Non-walking windows</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B12" t="n">
         <v>452</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Total duration (min)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>10.5</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Walking duration (min)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>3.0</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>── Energy (non-walking) ──</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Total energy Right (non-walk)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>75243.90</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Total energy Left (non-walk)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>80563.80</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Total energy combined (non-walk)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>155807.70</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>── Energy (walking) ──</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="B21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Total energy Right (walk)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>83250.50</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Total energy Left (walk)</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>44543.30</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>── Ratio R/L ──</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="B25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Mean ratio R/L</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>1.760</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Median ratio R/L</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>1.793</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>── Hourly breakdown ──</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="B29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Most energy-intense hour</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>11/03/2026 12:00</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Energy in most intense hour</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>155807.70</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Least energy-intense hour</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>11/03/2026 12:00</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Energy in least intense hour</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>155807.70</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>── Missing data periods ──</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="B35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Right wrist gaps (&gt;=10s)</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>0 gap(s)</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Left wrist gaps (&gt;=10s)</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>0 gap(s)</t>
         </is>

</xml_diff>